<commit_message>
checks related to the patient id columns
</commit_message>
<xml_diff>
--- a/tests/data/hidden_dates/iso8601.xlsx
+++ b/tests/data/hidden_dates/iso8601.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/hidden_dates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F088E032-CDFD-E848-AF43-C5AE7E088BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CD4716E-6CEF-264E-A4E6-A92B6431EE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4860" yWindow="-19480" windowWidth="23620" windowHeight="14320" xr2:uid="{056B165D-9BDB-444A-84F9-D21F3FE7A50D}"/>
+    <workbookView xWindow="0" yWindow="22200" windowWidth="28800" windowHeight="15600" xr2:uid="{056B165D-9BDB-444A-84F9-D21F3FE7A50D}"/>
   </bookViews>
   <sheets>
     <sheet name="args" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: structural checks (#129)
Co-authored-by: Peter LaValle <peter.lavalle@nhs.net>
</commit_message>
<xml_diff>
--- a/tests/data/hidden_dates/iso8601.xlsx
+++ b/tests/data/hidden_dates/iso8601.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/hidden_dates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F088E032-CDFD-E848-AF43-C5AE7E088BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CD4716E-6CEF-264E-A4E6-A92B6431EE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4860" yWindow="-19480" windowWidth="23620" windowHeight="14320" xr2:uid="{056B165D-9BDB-444A-84F9-D21F3FE7A50D}"/>
+    <workbookView xWindow="0" yWindow="22200" windowWidth="28800" windowHeight="15600" xr2:uid="{056B165D-9BDB-444A-84F9-D21F3FE7A50D}"/>
   </bookViews>
   <sheets>
     <sheet name="args" sheetId="1" r:id="rId1"/>

</xml_diff>